<commit_message>
refactor: update larga data
</commit_message>
<xml_diff>
--- a/examples/LargeDrugCombo_Goetz_Cancers_2024/tables/data__combo_fit_GR__Bliss_Score_GR.xlsx
+++ b/examples/LargeDrugCombo_Goetz_Cancers_2024/tables/data__combo_fit_GR__Bliss_Score_GR.xlsx
@@ -376,521 +376,521 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COLO 829</t>
+          <t>501A</t>
         </is>
       </c>
       <c r="B2">
-        <v>0.2404594183007559</v>
+        <v>0.1881678031921573</v>
       </c>
       <c r="C2">
-        <v>0.3374469991572689</v>
+        <v>0.2722821133307893</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SK-MEL-28</t>
+          <t>624 mel</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.1595205519647408</v>
+        <v>0.1388961711290195</v>
       </c>
       <c r="C3">
-        <v>0.1478844523164359</v>
+        <v>0.1268317642192261</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hs 695T</t>
+          <t>928 mel</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.1180026955852726</v>
+        <v>0.236702887201338</v>
       </c>
       <c r="C4">
-        <v>0.1315515443314705</v>
+        <v>0.1559901335230988</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MDA-MB-435</t>
+          <t>A-253</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.1096494534099406</v>
+        <v>0.03422622167501504</v>
       </c>
       <c r="C5">
-        <v>0.1580806584489273</v>
+        <v>0.2623027007916054</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>928 mel</t>
+          <t>A-375</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.236702887201338</v>
+        <v>0.04285682789925234</v>
       </c>
       <c r="C6">
-        <v>0.1559901335230988</v>
+        <v>0.09242661508550008</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>624 mel</t>
+          <t>A-431</t>
         </is>
       </c>
       <c r="B7">
-        <v>0.1388961711290195</v>
+        <v>0.2800043659887954</v>
       </c>
       <c r="C7">
-        <v>0.1268317642192261</v>
+        <v>0.5202340292211655</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RPMI-7951</t>
+          <t>A2058</t>
         </is>
       </c>
       <c r="B8">
-        <v>0.07761472076033336</v>
+        <v>0.03809980005181187</v>
       </c>
       <c r="C8">
-        <v>0.4210476561758792</v>
+        <v>0.0599290806193466</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G-361</t>
+          <t>A388</t>
         </is>
       </c>
       <c r="B9">
-        <v>0.232571734350346</v>
+        <v>0.2422222941626541</v>
       </c>
       <c r="C9">
-        <v>0.4550981689968096</v>
+        <v>0.375415538353883</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hs 294T</t>
+          <t>COLO 800</t>
         </is>
       </c>
       <c r="B10">
-        <v>0.1131996486706461</v>
+        <v>0.2776457396650376</v>
       </c>
       <c r="C10">
-        <v>0.1214313281893402</v>
+        <v>0.3346855811763834</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A-431</t>
+          <t>COLO 829</t>
         </is>
       </c>
       <c r="B11">
-        <v>0.2800043659887954</v>
+        <v>0.2404594183007559</v>
       </c>
       <c r="C11">
-        <v>0.5202340292211655</v>
+        <v>0.3374469991572689</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>A-375</t>
+          <t>COLO 849</t>
         </is>
       </c>
       <c r="B12">
-        <v>0.04285682789925234</v>
+        <v>0.3139455903849458</v>
       </c>
       <c r="C12">
-        <v>0.09242661508550008</v>
+        <v>0.2461447404374679</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>501A</t>
+          <t>COLO 857</t>
         </is>
       </c>
       <c r="B13">
-        <v>0.1881678031921573</v>
+        <v>0.06691517879227944</v>
       </c>
       <c r="C13">
-        <v>0.2722821133307893</v>
+        <v>0.1151258010449667</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SK-MEL-2</t>
+          <t>G-361</t>
         </is>
       </c>
       <c r="B14">
-        <v>0.0735107332959327</v>
+        <v>0.232571734350346</v>
       </c>
       <c r="C14">
-        <v>0.5624565926168456</v>
+        <v>0.4550981689968096</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MEL-JUSO</t>
+          <t>HCC1498</t>
         </is>
       </c>
       <c r="B15">
-        <v>0.09298243950058707</v>
+        <v>0.06908429954789519</v>
       </c>
       <c r="C15">
-        <v>0.3532076571060591</v>
+        <v>0.09582865787952938</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SK-MEL-30</t>
+          <t>HMY-1</t>
         </is>
       </c>
       <c r="B16">
-        <v>0.1216639948048155</v>
+        <v>0.07828483249764273</v>
       </c>
       <c r="C16">
-        <v>0.2830212132298639</v>
+        <v>0.08315347882790988</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hs 852.T</t>
+          <t>HSC-1</t>
         </is>
       </c>
       <c r="B17">
-        <v>0.1418265639222187</v>
+        <v>0.1619678758704838</v>
       </c>
       <c r="C17">
-        <v>0.8412627116271232</v>
+        <v>0.2889916503809022</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COLO 800</t>
+          <t>HT-144</t>
         </is>
       </c>
       <c r="B18">
-        <v>0.2776457396650376</v>
+        <v>0.2821392611206337</v>
       </c>
       <c r="C18">
-        <v>0.3346855811763834</v>
+        <v>0.3380219428882632</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SK-MEL-1</t>
+          <t>Hs 294T</t>
         </is>
       </c>
       <c r="B19">
-        <v>0.4339236821250738</v>
+        <v>0.1131996486706461</v>
       </c>
       <c r="C19">
-        <v>0.5992787936289778</v>
+        <v>0.1214313281893402</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>UACC-62</t>
+          <t>Hs 695T</t>
         </is>
       </c>
       <c r="B20">
-        <v>0.1888665876629614</v>
+        <v>0.1180026955852726</v>
       </c>
       <c r="C20">
-        <v>0.1596598257782368</v>
+        <v>0.1315515443314705</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SK-MEL-24</t>
+          <t>Hs 852.T</t>
         </is>
       </c>
       <c r="B21">
-        <v>0.2082649988489159</v>
+        <v>0.1418265639222187</v>
       </c>
       <c r="C21">
-        <v>0.2537034031905898</v>
+        <v>0.8412627116271232</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COLO 849</t>
+          <t>IGR-1</t>
         </is>
       </c>
       <c r="B22">
-        <v>0.3139455903849458</v>
+        <v>0.06515861683932005</v>
       </c>
       <c r="C22">
-        <v>0.2461447404374679</v>
+        <v>0.08733273736934667</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>A2058</t>
+          <t>IGR-39</t>
         </is>
       </c>
       <c r="B23">
-        <v>0.03809980005181187</v>
+        <v>0.05529167275896431</v>
       </c>
       <c r="C23">
-        <v>0.0599290806193466</v>
+        <v>0.1656012582989838</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SK23-mel</t>
+          <t>MDA-MB-435</t>
         </is>
       </c>
       <c r="B24">
-        <v>0.1653380085521752</v>
+        <v>0.1096494534099406</v>
       </c>
       <c r="C24">
-        <v>0.06403401388887586</v>
+        <v>0.1580806584489273</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>UCSD-242l</t>
+          <t>MEL-HO</t>
         </is>
       </c>
       <c r="B25">
-        <v>0.1382467749653447</v>
+        <v>0.2728166769712705</v>
       </c>
       <c r="C25">
-        <v>0.1044397968660734</v>
+        <v>0.2926772956119876</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MEL-HO</t>
+          <t>MEL-JUSO</t>
         </is>
       </c>
       <c r="B26">
-        <v>0.2728166769712705</v>
+        <v>0.09298243950058707</v>
       </c>
       <c r="C26">
-        <v>0.2926772956119876</v>
+        <v>0.3532076571060591</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>WM-266-4</t>
+          <t>MMAc</t>
         </is>
       </c>
       <c r="B27">
-        <v>0.2187681068328098</v>
+        <v>0.2349104432732611</v>
       </c>
       <c r="C27">
-        <v>0.1736589107776012</v>
+        <v>0.1958035413081212</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IGR-1</t>
+          <t>RPMI-7951</t>
         </is>
       </c>
       <c r="B28">
-        <v>0.06515861683932005</v>
+        <v>0.07761472076033336</v>
       </c>
       <c r="C28">
-        <v>0.08733273736934667</v>
+        <v>0.4210476561758792</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IGR-39</t>
+          <t>RVH-421</t>
         </is>
       </c>
       <c r="B29">
-        <v>0.05529167275896431</v>
+        <v>0.06594792561371243</v>
       </c>
       <c r="C29">
-        <v>0.1656012582989838</v>
+        <v>0.2070386240999933</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>COLO 857</t>
+          <t>SK-MEL-1</t>
         </is>
       </c>
       <c r="B30">
-        <v>0.06691517879227944</v>
+        <v>0.4339236821250738</v>
       </c>
       <c r="C30">
-        <v>0.1151258010449667</v>
+        <v>0.5992787936289778</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HMY-1</t>
+          <t>SK-MEL-2</t>
         </is>
       </c>
       <c r="B31">
-        <v>0.07828483249764273</v>
+        <v>0.0735107332959327</v>
       </c>
       <c r="C31">
-        <v>0.08315347882790988</v>
+        <v>0.5624565926168456</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MMAc</t>
+          <t>SK-MEL-24</t>
         </is>
       </c>
       <c r="B32">
-        <v>0.2349104432732611</v>
+        <v>0.2082649988489159</v>
       </c>
       <c r="C32">
-        <v>0.1958035413081212</v>
+        <v>0.2537034031905898</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SK-MEL-3</t>
+          <t>SK-MEL-28</t>
         </is>
       </c>
       <c r="B33">
-        <v>0.1679657833205432</v>
+        <v>0.1595205519647408</v>
       </c>
       <c r="C33">
-        <v>0.1362112024119674</v>
+        <v>0.1478844523164359</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RVH-421</t>
+          <t>SK-MEL-3</t>
         </is>
       </c>
       <c r="B34">
-        <v>0.06594792561371243</v>
+        <v>0.1679657833205432</v>
       </c>
       <c r="C34">
-        <v>0.2070386240999933</v>
+        <v>0.1362112024119674</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HSC-1</t>
+          <t>SK-MEL-30</t>
         </is>
       </c>
       <c r="B35">
-        <v>0.1619678758704838</v>
+        <v>0.1216639948048155</v>
       </c>
       <c r="C35">
-        <v>0.2889916503809022</v>
+        <v>0.2830212132298639</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>UACC-257</t>
+          <t>SK-MEL-31</t>
         </is>
       </c>
       <c r="B36">
-        <v>0.2025245249045179</v>
+        <v>0.1677646868715907</v>
       </c>
       <c r="C36">
-        <v>0.1642765376033153</v>
+        <v>0.1751180898584582</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SK-MEL-31</t>
+          <t>SK23-mel</t>
         </is>
       </c>
       <c r="B37">
-        <v>0.1677646868715907</v>
+        <v>0.1653380085521752</v>
       </c>
       <c r="C37">
-        <v>0.1751180898584582</v>
+        <v>0.06403401388887586</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HCC1498</t>
+          <t>UACC-257</t>
         </is>
       </c>
       <c r="B38">
-        <v>0.06908429954789519</v>
+        <v>0.2025245249045179</v>
       </c>
       <c r="C38">
-        <v>0.09582865787952938</v>
+        <v>0.1642765376033153</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>A-253</t>
+          <t>UACC-62</t>
         </is>
       </c>
       <c r="B39">
-        <v>0.03422622167501504</v>
+        <v>0.1888665876629614</v>
       </c>
       <c r="C39">
-        <v>0.2623027007916054</v>
+        <v>0.1596598257782368</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HT-144</t>
+          <t>UCSD-242l</t>
         </is>
       </c>
       <c r="B40">
-        <v>0.2821392611206337</v>
+        <v>0.1382467749653447</v>
       </c>
       <c r="C40">
-        <v>0.3380219428882632</v>
+        <v>0.1044397968660734</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>A388</t>
+          <t>WM-266-4</t>
         </is>
       </c>
       <c r="B41">
-        <v>0.2422222941626541</v>
+        <v>0.2187681068328098</v>
       </c>
       <c r="C41">
-        <v>0.375415538353883</v>
+        <v>0.1736589107776012</v>
       </c>
     </row>
   </sheetData>
@@ -918,7 +918,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COLO 829</t>
+          <t>501A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -930,7 +930,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SK-MEL-28</t>
+          <t>624 mel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -942,7 +942,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hs 695T</t>
+          <t>928 mel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -954,7 +954,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MDA-MB-435</t>
+          <t>A-253</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -966,7 +966,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>928 mel</t>
+          <t>A-375</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -978,7 +978,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>624 mel</t>
+          <t>A-431</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -990,7 +990,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RPMI-7951</t>
+          <t>A2058</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G-361</t>
+          <t>A388</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hs 294T</t>
+          <t>COLO 800</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A-431</t>
+          <t>COLO 829</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1038,7 +1038,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>A-375</t>
+          <t>COLO 849</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1050,7 +1050,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>501A</t>
+          <t>COLO 857</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1062,7 +1062,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SK-MEL-2</t>
+          <t>G-361</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MEL-JUSO</t>
+          <t>HCC1498</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1086,7 +1086,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SK-MEL-30</t>
+          <t>HMY-1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hs 852.T</t>
+          <t>HSC-1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1110,7 +1110,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COLO 800</t>
+          <t>HT-144</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1122,7 +1122,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SK-MEL-1</t>
+          <t>Hs 294T</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1134,7 +1134,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>UACC-62</t>
+          <t>Hs 695T</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1146,7 +1146,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SK-MEL-24</t>
+          <t>Hs 852.T</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1158,7 +1158,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COLO 849</t>
+          <t>IGR-1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1170,7 +1170,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>A2058</t>
+          <t>IGR-39</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1182,7 +1182,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SK23-mel</t>
+          <t>MDA-MB-435</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1194,7 +1194,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>UCSD-242l</t>
+          <t>MEL-HO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1206,7 +1206,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MEL-HO</t>
+          <t>MEL-JUSO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1218,7 +1218,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>WM-266-4</t>
+          <t>MMAc</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IGR-1</t>
+          <t>RPMI-7951</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1242,7 +1242,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IGR-39</t>
+          <t>RVH-421</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1254,7 +1254,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>COLO 857</t>
+          <t>SK-MEL-1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1266,7 +1266,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HMY-1</t>
+          <t>SK-MEL-2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1278,7 +1278,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MMAc</t>
+          <t>SK-MEL-24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1290,7 +1290,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SK-MEL-3</t>
+          <t>SK-MEL-28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1302,7 +1302,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RVH-421</t>
+          <t>SK-MEL-3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1314,7 +1314,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HSC-1</t>
+          <t>SK-MEL-30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>UACC-257</t>
+          <t>SK-MEL-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1338,7 +1338,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SK-MEL-31</t>
+          <t>SK23-mel</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1350,7 +1350,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HCC1498</t>
+          <t>UACC-257</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1362,7 +1362,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>A-253</t>
+          <t>UACC-62</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1374,7 +1374,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HT-144</t>
+          <t>UCSD-242l</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>A388</t>
+          <t>WM-266-4</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">

</xml_diff>